<commit_message>
sprint 16: actualizar REGISTRO y README al estado final; sumar Virk/Fawzy/Sharma a REFERENCIAS.xlsx
</commit_message>
<xml_diff>
--- a/REFERENCIAS.xlsx
+++ b/REFERENCIAS.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1804,6 +1804,141 @@
       <c r="K27" s="2" t="inlineStr">
         <is>
           <t>codegen</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Académico</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Non-programmers Assessing AI-Generated Code: A Case Study of Business Users Analyzing Data</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Virk, Liu</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="n">
+        <v>2025</v>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>VL/HCC 2025 (IEEE)</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>arXiv:2508.06484</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Virk2025_NonProgrammersAssessingAICode_VLHCC.pdf</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>sprint 16</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>virk2025nonprogrammers</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Académico</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>From Prompting to Verification: How Experience Shapes Vibe Coding Practices</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Fawzy, Tahir, Blincoe</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Preprint arXiv</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>arXiv:2605.24521</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Fawzy2026_PromptingToVerification_preprint.pdf</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>sprint 16</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>fawzy2026prompting</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Académico</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Feedback by Design: Understanding and Overcoming User Feedback Barriers in Conversational Agents</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Sharma, Zhang, Lee, Krishnan, Ren, Xiao, Li</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>CHI 2026</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>arXiv:2602.01405</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Sharma2026_FeedbackByDesign_CHI.pdf</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>sprint 16</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>sharma2026feedback</t>
         </is>
       </c>
     </row>

</xml_diff>